<commit_message>
chore: run 2026-03-26 18:09 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_26_03_2026.xlsx
+++ b/logs/Consolidado_26_03_2026.xlsx
@@ -638,7 +638,7 @@
         <v>151</v>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -6462,40 +6462,40 @@
       </c>
     </row>
     <row r="142">
-      <c r="A142" s="7" t="inlineStr">
-        <is>
-          <t>26/03/2026</t>
-        </is>
-      </c>
-      <c r="B142" s="7" t="inlineStr">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>26/03/2026</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C142" s="7" t="inlineStr">
+      <c r="C142" s="3" t="inlineStr">
         <is>
           <t>Ultra Serum Instantly Plumps SPF50+
 Protetor Solar Sérum Rosto AH+Niacinamida
 30 ml</t>
         </is>
       </c>
-      <c r="D142" s="7" t="inlineStr">
+      <c r="D142" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/ultra-serum-instantly-plumps-spf50-8784379.html</t>
         </is>
       </c>
-      <c r="E142" s="7" t="inlineStr"/>
-      <c r="F142" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G142" s="7" t="inlineStr">
+      <c r="E142" s="3" t="inlineStr"/>
+      <c r="F142" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G142" s="3" t="inlineStr">
         <is>
           <t>8784379</t>
         </is>
       </c>
-      <c r="H142" s="7" t="inlineStr">
+      <c r="H142" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>

</xml_diff>